<commit_message>
AI focus analysis added, updated output dataset
</commit_message>
<xml_diff>
--- a/data/keywords/topic_focus/keywords_topic_focus.xlsx
+++ b/data/keywords/topic_focus/keywords_topic_focus.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jojoa\OneDrive\Dokumente\OECD\RAnalysis\PRESS\data\keywords\topic_focus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED752876-6E6A-4453-BD4B-A11617D35A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81C64468-0E67-489A-B363-D95B2551EDC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AI" sheetId="7" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="45">
   <si>
     <t>id</t>
   </si>
@@ -46,12 +46,12 @@
     <t>fr</t>
   </si>
   <si>
+    <t>es</t>
+  </si>
+  <si>
     <t>de</t>
   </si>
   <si>
-    <t>es</t>
-  </si>
-  <si>
     <t>artificial intelligence</t>
   </si>
   <si>
@@ -112,14 +112,71 @@
     <t>genAI</t>
   </si>
   <si>
-    <t>LLM</t>
+    <t>natural language processing</t>
+  </si>
+  <si>
+    <t>neural network</t>
+  </si>
+  <si>
+    <t>computer vision</t>
+  </si>
+  <si>
+    <t>Sentiment Analysis</t>
+  </si>
+  <si>
+    <t>Chatbot</t>
+  </si>
+  <si>
+    <t>traitement du langage naturel</t>
+  </si>
+  <si>
+    <t>procesamiento del lenguaje natural</t>
+  </si>
+  <si>
+    <t>red neuronal</t>
+  </si>
+  <si>
+    <t>réseau de neurones</t>
+  </si>
+  <si>
+    <t>Neuronales Netzwerk</t>
+  </si>
+  <si>
+    <t>vision par ordinateur</t>
+  </si>
+  <si>
+    <t>visión por computador</t>
+  </si>
+  <si>
+    <t>visión artificial</t>
+  </si>
+  <si>
+    <t>análisis de sentimientos</t>
+  </si>
+  <si>
+    <t>analyse de sentiments</t>
+  </si>
+  <si>
+    <t>Sentiment-Analyse</t>
+  </si>
+  <si>
+    <t>agent conversationnel</t>
+  </si>
+  <si>
+    <t>bot conversacional</t>
+  </si>
+  <si>
+    <t>NLP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPT </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -146,11 +203,18 @@
       <sz val="11"/>
       <color theme="9" tint="-0.499984740745262"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="9" tint="-0.499984740745262"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -176,12 +240,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -472,106 +540,195 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A2" s="5">
+        <v>0</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A3" s="5">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A4" s="5">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A5" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
+      <c r="B5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A6" s="5">
+        <v>3</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A7" s="5">
+        <v>4</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="5"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A8" s="5">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="B8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A9" s="5">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="B9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="5"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A10" s="5">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="5"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A11" s="5">
         <v>7</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="B11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A12" s="5">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A5">
-        <v>3</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="4"/>
+      <c r="B12" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="5"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="4"/>
+      <c r="E13" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -580,7 +737,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34A530C6-6E1E-4869-A1CA-FDC34F8192D0}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
@@ -594,10 +751,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
@@ -613,7 +770,7 @@
       <c r="D2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="4"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3">
@@ -628,7 +785,15 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -646,6 +811,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9bae65c2-241c-418a-a37c-ddfb2f921707" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010033C2A0066C18BC4E9BE6DC4E41B0C07F" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="09e1717f508eb245191a7d70af1a5d50">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b" xmlns:ns3="9bae65c2-241c-418a-a37c-ddfb2f921707" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b81c025f9de5594d7b8cbb661cb82c62" ns2:_="" ns3:_="">
     <xsd:import namespace="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
@@ -906,17 +1082,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9bae65c2-241c-418a-a37c-ddfb2f921707" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{309E3272-FC41-444B-BA86-D1A5622D221C}">
   <ds:schemaRefs>
@@ -926,6 +1091,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E773F732-AD26-4990-9766-F75C55FCDDD2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
+    <ds:schemaRef ds:uri="9bae65c2-241c-418a-a37c-ddfb2f921707"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97FE3D86-31EC-465E-A8A6-6E0CEA7D99AC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -942,15 +1118,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E773F732-AD26-4990-9766-F75C55FCDDD2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
-    <ds:schemaRef ds:uri="9bae65c2-241c-418a-a37c-ddfb2f921707"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>